<commit_message>
Rename the app to 随心记账 (v0.8.7)
The README, the launcher label and the exported file names now agree. The
name had been written out five times -- app_name, both widget labels, two
ExportViewModel literals, the About and Settings cards, the widget's fallback
- so AppContainer now exposes it once and the export reads it from there.

The package stays com.pocketledger and the backup format tag stays
"pocketledger-backup": both are on disk in existing installs, and changing
either would orphan data rather than rename a product.
</commit_message>
<xml_diff>
--- a/tools/记账本文案.xlsx
+++ b/tools/记账本文案.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>app_name；导出与备份 · Prepare；导出与备份 · Prepare Backup 等5处</t>
+          <t>app_name；设置 · About Screen；桌面小组件 · Widget Body</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>记账本</t>
+          <t>随心记账</t>
         </is>
       </c>
       <c r="F4" s="5" t="n"/>
@@ -8258,7 +8258,7 @@
       </c>
       <c r="E300" s="7" t="inlineStr">
         <is>
-          <t>逐项说明记账本的各项功能</t>
+          <t>逐项说明随心记账的各项功能</t>
         </is>
       </c>
       <c r="F300" s="5" t="n"/>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="E353" s="7" t="inlineStr">
         <is>
-          <t>关于记账本</t>
+          <t>关于随心记账</t>
         </is>
       </c>
       <c r="F353" s="5" t="n"/>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E410" s="7" t="inlineStr">
         <is>
-          <t>记账本 · 本月</t>
+          <t>随心记账 · 本月</t>
         </is>
       </c>
       <c r="F410" s="5" t="n"/>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="E412" s="7" t="inlineStr">
         <is>
-          <t>记账本 · 本月概览</t>
+          <t>随心记账 · 本月概览</t>
         </is>
       </c>
       <c r="F412" s="5" t="n"/>
@@ -14043,7 +14043,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>备份来自更新的记账本（格式 v{version}），当前版本读不了。</t>
+          <t>备份来自更新的随心记账（格式 v{version}），当前版本读不了。</t>
         </is>
       </c>
       <c r="F6" s="5" t="n"/>
@@ -14069,7 +14069,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>这个文件不是记账本备份。</t>
+          <t>这个文件不是随心记账备份。</t>
         </is>
       </c>
       <c r="F7" s="5" t="n"/>
@@ -14095,7 +14095,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>这个文件不是记账本备份。</t>
+          <t>这个文件不是随心记账备份。</t>
         </is>
       </c>
       <c r="F8" s="5" t="n"/>

</xml_diff>